<commit_message>
modifiche funzionamento corretto + panda
</commit_message>
<xml_diff>
--- a/LaneFollowingControlWithSensorFusionAndLaneDetectionExample/tabellarisultati.xlsx
+++ b/LaneFollowingControlWithSensorFusionAndLaneDetectionExample/tabellarisultati.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="15" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="51" uniqueCount="9">
   <si>
     <t>Scenario</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t>Fitness_Hecate</t>
+  </si>
+  <si>
+    <t>Panda.m</t>
   </si>
 </sst>
 </file>
@@ -82,7 +85,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.81640625" customWidth="true"/>
@@ -139,10 +142,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C5" s="0">
-        <v>40.206713378310553</v>
+        <v>40.154626672007808</v>
       </c>
     </row>
     <row r="6">
@@ -150,10 +153,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C6" s="0">
-        <v>32.861443385021971</v>
+        <v>32.807297281769891</v>
       </c>
     </row>
     <row r="7">
@@ -161,10 +164,43 @@
         <v>3</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="0">
+        <v>25.629354485226827</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="0">
-        <v>24.180902039284554</v>
+      <c r="C8" s="0">
+        <v>40.202107995211016</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="0">
+        <v>32.861717388462139</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="0">
+        <v>6.5685656630786724</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
aggiunta di un veicolo e uno scenario
modificato inoltre il valore della distanza delle ruote posteriori e anteriori dal centro di gravità. Adesso corrisponde alla metà del passo del veicolo
</commit_message>
<xml_diff>
--- a/LaneFollowingControlWithSensorFusionAndLaneDetectionExample/tabellarisultati.xlsx
+++ b/LaneFollowingControlWithSensorFusionAndLaneDetectionExample/tabellarisultati.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="111" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="174" uniqueCount="14">
   <si>
     <t>Scenario</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>Anaconda</t>
+  </si>
+  <si>
+    <t>ACC_01_ISO_TargetDiscriminationTest</t>
+  </si>
+  <si>
+    <t>Colorado.m</t>
+  </si>
+  <si>
+    <t>A4.m</t>
   </si>
 </sst>
 </file>
@@ -91,11 +100,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.81640625" customWidth="true"/>
-    <col min="2" max="2" width="9.6328125" customWidth="true"/>
+    <col min="2" max="2" width="10.7265625" customWidth="true"/>
     <col min="3" max="3" width="13.36328125" customWidth="true"/>
   </cols>
   <sheetData>
@@ -118,7 +127,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="0">
-        <v>40.139505642076038</v>
+        <v>40.145833171463458</v>
       </c>
     </row>
     <row r="3">
@@ -129,7 +138,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="0">
-        <v>32.778807803704908</v>
+        <v>32.809569263513914</v>
       </c>
     </row>
     <row r="4">
@@ -140,7 +149,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="0">
-        <v>24.749103030307012</v>
+        <v>22.017838928658158</v>
       </c>
     </row>
     <row r="5">
@@ -151,7 +160,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="0">
-        <v>33.208963129466035</v>
+        <v>33.229882279081274</v>
       </c>
     </row>
     <row r="6">
@@ -162,117 +171,282 @@
         <v>5</v>
       </c>
       <c r="C6" s="0">
-        <v>30.94702999784662</v>
+        <v>30.755956303763455</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C7" s="0">
-        <v>40.154626672007808</v>
+        <v>49.802777927196701</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="0">
-        <v>32.807297281769891</v>
+        <v>40.129656025454075</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="0">
-        <v>25.629354485226827</v>
+        <v>32.798168031389402</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="0">
-        <v>33.050151997114838</v>
+        <v>26.568991997452919</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="0">
-        <v>30.962740151133488</v>
+        <v>33.203020544767703</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C12" s="0">
-        <v>40.202107995211016</v>
+        <v>30.96665412533568</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C13" s="0">
-        <v>32.861717388462139</v>
+        <v>50.198912485855551</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B14" s="0" t="s">
         <v>6</v>
       </c>
       <c r="C14" s="0">
-        <v>6.5685656630786724</v>
+        <v>40.198763756774866</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>6</v>
       </c>
       <c r="C15" s="0">
-        <v>33.3162792201149</v>
+        <v>30.308346551545299</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="0">
+        <v>22.168889762644177</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="0">
+        <v>27.398325126422456</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="0">
-        <v>30.937433890130642</v>
+      <c r="B18" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="0">
+        <v>30.966712812186238</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="0">
+        <v>49.545376555653938</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="0">
+        <v>40.162021071193585</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="0">
+        <v>32.892167691786639</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="0">
+        <v>10.439338970348871</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="0">
+        <v>33.195935931757063</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="0">
+        <v>30.952523680957086</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="0">
+        <v>49.822874350175752</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="0">
+        <v>40.17364891713968</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="0">
+        <v>32.843859309996049</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="0">
+        <v>25.543714011477746</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="0">
+        <v>4.9667712560198929</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="0">
+        <v>30.975353459770574</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="0">
+        <v>50.530793849331033</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tutti scenari funzionanti + aggiunta informazione tempo
</commit_message>
<xml_diff>
--- a/LaneFollowingControlWithSensorFusionAndLaneDetectionExample/tabellarisultati.xlsx
+++ b/LaneFollowingControlWithSensorFusionAndLaneDetectionExample/tabellarisultati.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="404" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="547" uniqueCount="21">
   <si>
     <t>Scenario</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>FrenataBrusca</t>
+  </si>
+  <si>
+    <t>Highway_double_target</t>
   </si>
 </sst>
 </file>
@@ -227,13 +230,13 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="0">
-        <v>3.73397812150254</v>
+        <v>39.82686101201962</v>
       </c>
     </row>
     <row r="11">
@@ -337,13 +340,13 @@
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B20" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="0">
-        <v>4.2659087417113692</v>
+        <v>43.568877088224845</v>
       </c>
     </row>
     <row r="21">
@@ -447,13 +450,13 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B30" s="0" t="s">
         <v>6</v>
       </c>
       <c r="C30" s="0">
-        <v>0.30454350796696161</v>
+        <v>43.668292538098775</v>
       </c>
     </row>
     <row r="31">
@@ -557,13 +560,13 @@
     </row>
     <row r="40">
       <c r="A40" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B40" s="0" t="s">
         <v>12</v>
       </c>
       <c r="C40" s="0">
-        <v>-2.5803514835608903</v>
+        <v>43.037552396657858</v>
       </c>
     </row>
     <row r="41">
@@ -667,13 +670,13 @@
     </row>
     <row r="50">
       <c r="A50" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B50" s="0" t="s">
         <v>13</v>
       </c>
       <c r="C50" s="0">
-        <v>-1.0624538531275665</v>
+        <v>44.878457488199906</v>
       </c>
     </row>
     <row r="51">
@@ -777,13 +780,13 @@
     </row>
     <row r="60">
       <c r="A60" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B60" s="0" t="s">
         <v>14</v>
       </c>
       <c r="C60" s="0">
-        <v>3.0316564853648114</v>
+        <v>45.267474773366743</v>
       </c>
     </row>
     <row r="61">
@@ -887,13 +890,13 @@
     </row>
     <row r="70">
       <c r="A70" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B70" s="0" t="s">
         <v>15</v>
       </c>
       <c r="C70" s="0">
-        <v>-0.55031151546863377</v>
+        <v>43.77004414281123</v>
       </c>
     </row>
     <row r="71">

</xml_diff>